<commit_message>
upload file table show
</commit_message>
<xml_diff>
--- a/Cygnux.LSP.Backend/Cygnux.LSP.Api/Uploads/Docket_Import.xlsx
+++ b/Cygnux.LSP.Backend/Cygnux.LSP.Api/Uploads/Docket_Import.xlsx
@@ -29,10 +29,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
-    <t>LspName</t>
+    <t>LSPName</t>
   </si>
   <si>
-    <t>DocketNO</t>
+    <t>DocketNo</t>
   </si>
   <si>
     <t>InvoiceNo</t>
@@ -41,16 +41,16 @@
     <t>Date</t>
   </si>
   <si>
-    <t>From</t>
+    <t>FromLocation</t>
   </si>
   <si>
-    <t>TO</t>
+    <t>ToLocation</t>
   </si>
   <si>
     <t>Quantity</t>
   </si>
   <si>
-    <t>Mode of Transporter</t>
+    <t>ModeOfTransporter</t>
   </si>
 </sst>
 </file>

</xml_diff>